<commit_message>
feat(datos-clientes): add module datos_clientes with endpoints, startup migration, and tests
</commit_message>
<xml_diff>
--- a/app/templates/Recepciones/F-LEM-P-01.13 V01 RECEP DE MUESTRA.XLSX
+++ b/app/templates/Recepciones/F-LEM-P-01.13 V01 RECEP DE MUESTRA.XLSX
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27928"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B044A5F6-9998-4EDE-9901-513CC97CEA4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{502F41CE-D5CC-4CC2-BE31-1CD460014CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -79,9 +79,6 @@
     <t>N°</t>
   </si>
   <si>
-    <t>* No llenar la zona sombreada</t>
-  </si>
-  <si>
     <t>RECEPCIÓN N°:</t>
   </si>
   <si>
@@ -211,6 +208,9 @@
   </si>
   <si>
     <t>RECEPCIÓN DE MUESTRA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">* No llenar la zona sombreada / albañileria se solicita marca y tipo </t>
   </si>
 </sst>
 </file>
@@ -586,6 +586,105 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -594,12 +693,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -610,99 +703,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1158,21 +1158,21 @@
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
       <c r="D1" s="5"/>
-      <c r="E1" s="81" t="s">
-        <v>59</v>
-      </c>
-      <c r="F1" s="81"/>
-      <c r="G1" s="81"/>
-      <c r="H1" s="81"/>
-      <c r="I1" s="81"/>
-      <c r="J1" s="81"/>
-      <c r="K1" s="81"/>
-      <c r="L1" s="77" t="s">
+      <c r="E1" s="67" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="63" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="78"/>
+      <c r="M1" s="64"/>
       <c r="N1" s="44" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O1" s="40"/>
     </row>
@@ -1181,17 +1181,17 @@
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
       <c r="D2" s="8"/>
-      <c r="E2" s="81"/>
-      <c r="F2" s="81"/>
-      <c r="G2" s="81"/>
-      <c r="H2" s="81"/>
-      <c r="I2" s="81"/>
-      <c r="J2" s="81"/>
-      <c r="K2" s="81"/>
-      <c r="L2" s="79" t="s">
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="65" t="s">
         <v>7</v>
       </c>
-      <c r="M2" s="80"/>
+      <c r="M2" s="66"/>
       <c r="N2" s="45">
         <v>2</v>
       </c>
@@ -1202,17 +1202,17 @@
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
       <c r="D3" s="8"/>
-      <c r="E3" s="81"/>
-      <c r="F3" s="81"/>
-      <c r="G3" s="81"/>
-      <c r="H3" s="81"/>
-      <c r="I3" s="81"/>
-      <c r="J3" s="81"/>
-      <c r="K3" s="81"/>
-      <c r="L3" s="79" t="s">
+      <c r="E3" s="67"/>
+      <c r="F3" s="67"/>
+      <c r="G3" s="67"/>
+      <c r="H3" s="67"/>
+      <c r="I3" s="67"/>
+      <c r="J3" s="67"/>
+      <c r="K3" s="67"/>
+      <c r="L3" s="65" t="s">
         <v>10</v>
       </c>
-      <c r="M3" s="80"/>
+      <c r="M3" s="66"/>
       <c r="N3" s="46">
         <v>46255</v>
       </c>
@@ -1223,17 +1223,17 @@
       <c r="B4" s="10"/>
       <c r="C4" s="10"/>
       <c r="D4" s="11"/>
-      <c r="E4" s="81"/>
-      <c r="F4" s="81"/>
-      <c r="G4" s="81"/>
-      <c r="H4" s="81"/>
-      <c r="I4" s="81"/>
-      <c r="J4" s="81"/>
-      <c r="K4" s="81"/>
-      <c r="L4" s="77" t="s">
+      <c r="E4" s="67"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="67"/>
+      <c r="H4" s="67"/>
+      <c r="I4" s="67"/>
+      <c r="J4" s="67"/>
+      <c r="K4" s="67"/>
+      <c r="L4" s="63" t="s">
         <v>8</v>
       </c>
-      <c r="M4" s="78"/>
+      <c r="M4" s="64"/>
       <c r="N4" s="44" t="s">
         <v>9</v>
       </c>
@@ -1257,52 +1257,52 @@
       <c r="O5" s="12"/>
     </row>
     <row r="6" spans="1:19" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="66" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="66"/>
+      <c r="A6" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="75"/>
       <c r="C6" s="7"/>
       <c r="D6" s="39">
         <v>0</v>
       </c>
       <c r="E6" s="13"/>
       <c r="F6" s="37" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G6" s="7"/>
       <c r="I6" s="23">
         <v>0</v>
       </c>
-      <c r="K6" s="82" t="s">
-        <v>35</v>
+      <c r="K6" s="68" t="s">
+        <v>34</v>
       </c>
       <c r="L6" s="38" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="M6" s="27" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="74" t="s">
-        <v>30</v>
-      </c>
-      <c r="B7" s="74"/>
+      <c r="A7" s="76" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="76"/>
       <c r="C7" s="7"/>
       <c r="D7" s="39">
         <v>0</v>
       </c>
       <c r="E7" s="13"/>
       <c r="F7" s="37" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G7" s="13"/>
       <c r="I7" s="23">
         <v>0</v>
       </c>
-      <c r="K7" s="82"/>
+      <c r="K7" s="68"/>
       <c r="L7" s="38" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M7" s="27"/>
     </row>
@@ -1325,7 +1325,7 @@
     </row>
     <row r="9" spans="1:19" ht="19.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" s="16"/>
       <c r="C9" s="17"/>
@@ -1345,23 +1345,23 @@
       <c r="C10" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D10" s="56"/>
-      <c r="E10" s="56"/>
-      <c r="F10" s="56"/>
-      <c r="G10" s="56"/>
-      <c r="H10" s="56"/>
-      <c r="I10" s="56"/>
-      <c r="J10" s="56"/>
-      <c r="K10" s="56"/>
-      <c r="L10" s="56"/>
-      <c r="M10" s="56"/>
-      <c r="N10" s="56"/>
-      <c r="P10" s="53" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q10" s="53"/>
-      <c r="R10" s="53"/>
-      <c r="S10" s="53"/>
+      <c r="D10" s="69"/>
+      <c r="E10" s="69"/>
+      <c r="F10" s="69"/>
+      <c r="G10" s="69"/>
+      <c r="H10" s="69"/>
+      <c r="I10" s="69"/>
+      <c r="J10" s="69"/>
+      <c r="K10" s="69"/>
+      <c r="L10" s="69"/>
+      <c r="M10" s="69"/>
+      <c r="N10" s="69"/>
+      <c r="P10" s="81" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q10" s="81"/>
+      <c r="R10" s="81"/>
+      <c r="S10" s="81"/>
     </row>
     <row r="11" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
@@ -1371,21 +1371,21 @@
       <c r="C11" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D11" s="56"/>
-      <c r="E11" s="56"/>
-      <c r="F11" s="56"/>
-      <c r="G11" s="56"/>
-      <c r="H11" s="56"/>
-      <c r="I11" s="56"/>
-      <c r="J11" s="56"/>
-      <c r="K11" s="56"/>
-      <c r="L11" s="56"/>
-      <c r="M11" s="56"/>
-      <c r="N11" s="56"/>
-      <c r="P11" s="53"/>
-      <c r="Q11" s="53"/>
-      <c r="R11" s="53"/>
-      <c r="S11" s="53"/>
+      <c r="D11" s="69"/>
+      <c r="E11" s="69"/>
+      <c r="F11" s="69"/>
+      <c r="G11" s="69"/>
+      <c r="H11" s="69"/>
+      <c r="I11" s="69"/>
+      <c r="J11" s="69"/>
+      <c r="K11" s="69"/>
+      <c r="L11" s="69"/>
+      <c r="M11" s="69"/>
+      <c r="N11" s="69"/>
+      <c r="P11" s="81"/>
+      <c r="Q11" s="81"/>
+      <c r="R11" s="81"/>
+      <c r="S11" s="81"/>
     </row>
     <row r="12" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
@@ -1395,21 +1395,21 @@
       <c r="C12" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D12" s="55"/>
-      <c r="E12" s="55"/>
-      <c r="F12" s="55"/>
-      <c r="G12" s="55"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="55"/>
-      <c r="J12" s="55"/>
-      <c r="K12" s="55"/>
-      <c r="L12" s="55"/>
-      <c r="M12" s="55"/>
-      <c r="N12" s="55"/>
-      <c r="P12" s="53"/>
-      <c r="Q12" s="53"/>
-      <c r="R12" s="53"/>
-      <c r="S12" s="53"/>
+      <c r="D12" s="52"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="52"/>
+      <c r="I12" s="52"/>
+      <c r="J12" s="52"/>
+      <c r="K12" s="52"/>
+      <c r="L12" s="52"/>
+      <c r="M12" s="52"/>
+      <c r="N12" s="52"/>
+      <c r="P12" s="81"/>
+      <c r="Q12" s="81"/>
+      <c r="R12" s="81"/>
+      <c r="S12" s="81"/>
     </row>
     <row r="13" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
@@ -1419,21 +1419,21 @@
       <c r="C13" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D13" s="55"/>
-      <c r="E13" s="55"/>
-      <c r="F13" s="55"/>
-      <c r="G13" s="55"/>
-      <c r="H13" s="55"/>
-      <c r="I13" s="55"/>
-      <c r="J13" s="55"/>
-      <c r="K13" s="55"/>
-      <c r="L13" s="55"/>
-      <c r="M13" s="55"/>
-      <c r="N13" s="55"/>
-      <c r="P13" s="53"/>
-      <c r="Q13" s="53"/>
-      <c r="R13" s="53"/>
-      <c r="S13" s="53"/>
+      <c r="D13" s="52"/>
+      <c r="E13" s="52"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="52"/>
+      <c r="I13" s="52"/>
+      <c r="J13" s="52"/>
+      <c r="K13" s="52"/>
+      <c r="L13" s="52"/>
+      <c r="M13" s="52"/>
+      <c r="N13" s="52"/>
+      <c r="P13" s="81"/>
+      <c r="Q13" s="81"/>
+      <c r="R13" s="81"/>
+      <c r="S13" s="81"/>
     </row>
     <row r="14" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
@@ -1443,23 +1443,23 @@
       <c r="C14" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D14" s="55"/>
-      <c r="E14" s="55"/>
-      <c r="F14" s="55"/>
-      <c r="G14" s="55"/>
-      <c r="H14" s="55"/>
-      <c r="I14" s="55"/>
+      <c r="D14" s="52"/>
+      <c r="E14" s="52"/>
+      <c r="F14" s="52"/>
+      <c r="G14" s="52"/>
+      <c r="H14" s="52"/>
+      <c r="I14" s="52"/>
       <c r="J14" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="K14" s="55"/>
-      <c r="L14" s="55"/>
-      <c r="M14" s="55"/>
-      <c r="N14" s="55"/>
-      <c r="P14" s="53"/>
-      <c r="Q14" s="53"/>
-      <c r="R14" s="53"/>
-      <c r="S14" s="53"/>
+        <v>17</v>
+      </c>
+      <c r="K14" s="52"/>
+      <c r="L14" s="52"/>
+      <c r="M14" s="52"/>
+      <c r="N14" s="52"/>
+      <c r="P14" s="81"/>
+      <c r="Q14" s="81"/>
+      <c r="R14" s="81"/>
+      <c r="S14" s="81"/>
     </row>
     <row r="15" spans="1:19" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="25" t="s">
@@ -1488,47 +1488,47 @@
       <c r="C16" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D16" s="56"/>
-      <c r="E16" s="56"/>
-      <c r="F16" s="56"/>
-      <c r="G16" s="56"/>
-      <c r="H16" s="56"/>
-      <c r="I16" s="56"/>
-      <c r="J16" s="56"/>
-      <c r="K16" s="56"/>
-      <c r="L16" s="56"/>
-      <c r="M16" s="56"/>
-      <c r="N16" s="56"/>
-      <c r="P16" s="53" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q16" s="53"/>
-      <c r="R16" s="53"/>
-      <c r="S16" s="53"/>
+      <c r="D16" s="69"/>
+      <c r="E16" s="69"/>
+      <c r="F16" s="69"/>
+      <c r="G16" s="69"/>
+      <c r="H16" s="69"/>
+      <c r="I16" s="69"/>
+      <c r="J16" s="69"/>
+      <c r="K16" s="69"/>
+      <c r="L16" s="69"/>
+      <c r="M16" s="69"/>
+      <c r="N16" s="69"/>
+      <c r="P16" s="81" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q16" s="81"/>
+      <c r="R16" s="81"/>
+      <c r="S16" s="81"/>
     </row>
     <row r="17" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="48" t="s">
+      <c r="A17" s="78" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="48"/>
+      <c r="B17" s="78"/>
       <c r="C17" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D17" s="56"/>
-      <c r="E17" s="56"/>
-      <c r="F17" s="56"/>
-      <c r="G17" s="56"/>
-      <c r="H17" s="56"/>
-      <c r="I17" s="56"/>
-      <c r="J17" s="56"/>
-      <c r="K17" s="56"/>
-      <c r="L17" s="56"/>
-      <c r="M17" s="56"/>
-      <c r="N17" s="56"/>
-      <c r="P17" s="53"/>
-      <c r="Q17" s="53"/>
-      <c r="R17" s="53"/>
-      <c r="S17" s="53"/>
+      <c r="D17" s="69"/>
+      <c r="E17" s="69"/>
+      <c r="F17" s="69"/>
+      <c r="G17" s="69"/>
+      <c r="H17" s="69"/>
+      <c r="I17" s="69"/>
+      <c r="J17" s="69"/>
+      <c r="K17" s="69"/>
+      <c r="L17" s="69"/>
+      <c r="M17" s="69"/>
+      <c r="N17" s="69"/>
+      <c r="P17" s="81"/>
+      <c r="Q17" s="81"/>
+      <c r="R17" s="81"/>
+      <c r="S17" s="81"/>
     </row>
     <row r="18" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
@@ -1538,21 +1538,21 @@
       <c r="C18" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D18" s="55"/>
-      <c r="E18" s="55"/>
-      <c r="F18" s="55"/>
-      <c r="G18" s="55"/>
-      <c r="H18" s="55"/>
-      <c r="I18" s="55"/>
-      <c r="J18" s="55"/>
-      <c r="K18" s="55"/>
-      <c r="L18" s="55"/>
-      <c r="M18" s="55"/>
-      <c r="N18" s="55"/>
-      <c r="P18" s="53"/>
-      <c r="Q18" s="53"/>
-      <c r="R18" s="53"/>
-      <c r="S18" s="53"/>
+      <c r="D18" s="52"/>
+      <c r="E18" s="52"/>
+      <c r="F18" s="52"/>
+      <c r="G18" s="52"/>
+      <c r="H18" s="52"/>
+      <c r="I18" s="52"/>
+      <c r="J18" s="52"/>
+      <c r="K18" s="52"/>
+      <c r="L18" s="52"/>
+      <c r="M18" s="52"/>
+      <c r="N18" s="52"/>
+      <c r="P18" s="81"/>
+      <c r="Q18" s="81"/>
+      <c r="R18" s="81"/>
+      <c r="S18" s="81"/>
     </row>
     <row r="19" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
@@ -1562,25 +1562,25 @@
       <c r="C19" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D19" s="55"/>
-      <c r="E19" s="55"/>
-      <c r="F19" s="55"/>
-      <c r="G19" s="55"/>
-      <c r="H19" s="55"/>
-      <c r="I19" s="55"/>
-      <c r="J19" s="55"/>
-      <c r="K19" s="55"/>
-      <c r="L19" s="55"/>
-      <c r="M19" s="55"/>
-      <c r="N19" s="55"/>
-      <c r="P19" s="53"/>
-      <c r="Q19" s="53"/>
-      <c r="R19" s="53"/>
-      <c r="S19" s="53"/>
+      <c r="D19" s="52"/>
+      <c r="E19" s="52"/>
+      <c r="F19" s="52"/>
+      <c r="G19" s="52"/>
+      <c r="H19" s="52"/>
+      <c r="I19" s="52"/>
+      <c r="J19" s="52"/>
+      <c r="K19" s="52"/>
+      <c r="L19" s="52"/>
+      <c r="M19" s="52"/>
+      <c r="N19" s="52"/>
+      <c r="P19" s="81"/>
+      <c r="Q19" s="81"/>
+      <c r="R19" s="81"/>
+      <c r="S19" s="81"/>
     </row>
     <row r="20" spans="1:19" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>16</v>
+        <v>59</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -1600,27 +1600,27 @@
         <v>15</v>
       </c>
       <c r="B21" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="C21" s="50" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="61" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" s="62"/>
+      <c r="E21" s="62"/>
+      <c r="F21" s="62"/>
+      <c r="G21" s="80"/>
+      <c r="H21" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="I21" s="61" t="s">
         <v>21</v>
       </c>
-      <c r="D21" s="51"/>
-      <c r="E21" s="51"/>
-      <c r="F21" s="51"/>
-      <c r="G21" s="52"/>
-      <c r="H21" s="30" t="s">
-        <v>58</v>
-      </c>
-      <c r="I21" s="50" t="s">
-        <v>22</v>
-      </c>
-      <c r="J21" s="51"/>
-      <c r="K21" s="51"/>
-      <c r="L21" s="51"/>
+      <c r="J21" s="62"/>
+      <c r="K21" s="62"/>
+      <c r="L21" s="62"/>
       <c r="M21" s="31"/>
       <c r="N21" s="29" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="O21" s="41"/>
     </row>
@@ -1629,230 +1629,230 @@
         <v>1</v>
       </c>
       <c r="B22" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="C22" s="67" t="s">
+        <v>52</v>
+      </c>
+      <c r="C22" s="51" t="s">
+        <v>54</v>
+      </c>
+      <c r="D22" s="52"/>
+      <c r="E22" s="52"/>
+      <c r="F22" s="53" t="s">
         <v>55</v>
       </c>
-      <c r="D22" s="55"/>
-      <c r="E22" s="55"/>
-      <c r="F22" s="72" t="s">
-        <v>56</v>
-      </c>
-      <c r="G22" s="73"/>
+      <c r="G22" s="54"/>
       <c r="H22" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="I22" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J22" s="64"/>
-      <c r="K22" s="64"/>
-      <c r="L22" s="64"/>
-      <c r="M22" s="65"/>
+        <v>38</v>
+      </c>
+      <c r="I22" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J22" s="71"/>
+      <c r="K22" s="71"/>
+      <c r="L22" s="71"/>
+      <c r="M22" s="72"/>
       <c r="N22" s="35" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="O22" s="42"/>
     </row>
     <row r="23" spans="1:19" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="32"/>
       <c r="B23" s="33"/>
-      <c r="C23" s="57" t="s">
-        <v>26</v>
-      </c>
-      <c r="D23" s="58"/>
-      <c r="E23" s="58"/>
-      <c r="F23" s="70" t="s">
-        <v>56</v>
-      </c>
-      <c r="G23" s="71"/>
+      <c r="C23" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="D23" s="48"/>
+      <c r="E23" s="48"/>
+      <c r="F23" s="55" t="s">
+        <v>55</v>
+      </c>
+      <c r="G23" s="56"/>
       <c r="H23" s="34" t="s">
-        <v>40</v>
-      </c>
-      <c r="I23" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J23" s="64"/>
-      <c r="K23" s="64"/>
-      <c r="L23" s="64"/>
-      <c r="M23" s="65"/>
+        <v>39</v>
+      </c>
+      <c r="I23" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J23" s="71"/>
+      <c r="K23" s="71"/>
+      <c r="L23" s="71"/>
+      <c r="M23" s="72"/>
       <c r="N23" s="35" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="O23" s="42"/>
     </row>
     <row r="24" spans="1:19" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="32"/>
       <c r="B24" s="33"/>
-      <c r="C24" s="61" t="s">
-        <v>29</v>
-      </c>
-      <c r="D24" s="62"/>
-      <c r="E24" s="62"/>
-      <c r="F24" s="68" t="s">
-        <v>56</v>
-      </c>
-      <c r="G24" s="69"/>
+      <c r="C24" s="57" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" s="58"/>
+      <c r="E24" s="58"/>
+      <c r="F24" s="59" t="s">
+        <v>55</v>
+      </c>
+      <c r="G24" s="60"/>
       <c r="H24" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="I24" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J24" s="64"/>
-      <c r="K24" s="64"/>
-      <c r="L24" s="64"/>
-      <c r="M24" s="65"/>
+        <v>40</v>
+      </c>
+      <c r="I24" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J24" s="71"/>
+      <c r="K24" s="71"/>
+      <c r="L24" s="71"/>
+      <c r="M24" s="72"/>
       <c r="N24" s="35" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="O24" s="42"/>
     </row>
     <row r="25" spans="1:19" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="32"/>
       <c r="B25" s="33"/>
-      <c r="C25" s="57" t="s">
-        <v>28</v>
-      </c>
-      <c r="D25" s="58"/>
-      <c r="E25" s="58"/>
-      <c r="F25" s="59" t="s">
-        <v>56</v>
-      </c>
-      <c r="G25" s="60"/>
+      <c r="C25" s="47" t="s">
+        <v>27</v>
+      </c>
+      <c r="D25" s="48"/>
+      <c r="E25" s="48"/>
+      <c r="F25" s="49" t="s">
+        <v>55</v>
+      </c>
+      <c r="G25" s="50"/>
       <c r="H25" s="34" t="s">
-        <v>42</v>
-      </c>
-      <c r="I25" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J25" s="64"/>
-      <c r="K25" s="64"/>
-      <c r="L25" s="64"/>
-      <c r="M25" s="65"/>
+        <v>41</v>
+      </c>
+      <c r="I25" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J25" s="71"/>
+      <c r="K25" s="71"/>
+      <c r="L25" s="71"/>
+      <c r="M25" s="72"/>
       <c r="N25" s="35"/>
       <c r="O25" s="42"/>
     </row>
     <row r="26" spans="1:19" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="32"/>
       <c r="B26" s="33"/>
-      <c r="C26" s="57"/>
-      <c r="D26" s="58"/>
-      <c r="E26" s="58"/>
-      <c r="F26" s="59"/>
-      <c r="G26" s="60"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="48"/>
+      <c r="E26" s="48"/>
+      <c r="F26" s="49"/>
+      <c r="G26" s="50"/>
       <c r="H26" s="34" t="s">
-        <v>43</v>
-      </c>
-      <c r="I26" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J26" s="64"/>
-      <c r="K26" s="64"/>
-      <c r="L26" s="64"/>
-      <c r="M26" s="65"/>
+        <v>42</v>
+      </c>
+      <c r="I26" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J26" s="71"/>
+      <c r="K26" s="71"/>
+      <c r="L26" s="71"/>
+      <c r="M26" s="72"/>
       <c r="N26" s="35"/>
       <c r="O26" s="42"/>
     </row>
     <row r="27" spans="1:19" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="32"/>
       <c r="B27" s="33"/>
-      <c r="C27" s="57"/>
-      <c r="D27" s="58"/>
-      <c r="E27" s="58"/>
-      <c r="F27" s="59"/>
-      <c r="G27" s="60"/>
+      <c r="C27" s="47"/>
+      <c r="D27" s="48"/>
+      <c r="E27" s="48"/>
+      <c r="F27" s="49"/>
+      <c r="G27" s="50"/>
       <c r="H27" s="34" t="s">
-        <v>44</v>
-      </c>
-      <c r="I27" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J27" s="64"/>
-      <c r="K27" s="64"/>
-      <c r="L27" s="64"/>
-      <c r="M27" s="65"/>
+        <v>43</v>
+      </c>
+      <c r="I27" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J27" s="71"/>
+      <c r="K27" s="71"/>
+      <c r="L27" s="71"/>
+      <c r="M27" s="72"/>
       <c r="N27" s="35"/>
       <c r="O27" s="42"/>
     </row>
     <row r="28" spans="1:19" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="32"/>
       <c r="B28" s="33"/>
-      <c r="C28" s="57"/>
-      <c r="D28" s="58"/>
-      <c r="E28" s="58"/>
-      <c r="F28" s="59"/>
-      <c r="G28" s="60"/>
+      <c r="C28" s="47"/>
+      <c r="D28" s="48"/>
+      <c r="E28" s="48"/>
+      <c r="F28" s="49"/>
+      <c r="G28" s="50"/>
       <c r="H28" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="I28" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J28" s="64"/>
-      <c r="K28" s="64"/>
-      <c r="L28" s="64"/>
-      <c r="M28" s="65"/>
+        <v>44</v>
+      </c>
+      <c r="I28" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J28" s="71"/>
+      <c r="K28" s="71"/>
+      <c r="L28" s="71"/>
+      <c r="M28" s="72"/>
       <c r="N28" s="35"/>
       <c r="O28" s="42"/>
     </row>
     <row r="29" spans="1:19" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="32"/>
       <c r="B29" s="33"/>
-      <c r="C29" s="57"/>
-      <c r="D29" s="58"/>
-      <c r="E29" s="58"/>
-      <c r="F29" s="59"/>
-      <c r="G29" s="60"/>
+      <c r="C29" s="47"/>
+      <c r="D29" s="48"/>
+      <c r="E29" s="48"/>
+      <c r="F29" s="49"/>
+      <c r="G29" s="50"/>
       <c r="H29" s="34" t="s">
-        <v>46</v>
-      </c>
-      <c r="I29" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J29" s="64"/>
-      <c r="K29" s="64"/>
-      <c r="L29" s="64"/>
-      <c r="M29" s="65"/>
+        <v>45</v>
+      </c>
+      <c r="I29" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J29" s="71"/>
+      <c r="K29" s="71"/>
+      <c r="L29" s="71"/>
+      <c r="M29" s="72"/>
       <c r="N29" s="35"/>
       <c r="O29" s="42"/>
     </row>
     <row r="30" spans="1:19" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="32"/>
       <c r="B30" s="33"/>
-      <c r="C30" s="57"/>
-      <c r="D30" s="58"/>
-      <c r="E30" s="58"/>
-      <c r="F30" s="59"/>
-      <c r="G30" s="60"/>
+      <c r="C30" s="47"/>
+      <c r="D30" s="48"/>
+      <c r="E30" s="48"/>
+      <c r="F30" s="49"/>
+      <c r="G30" s="50"/>
       <c r="H30" s="34" t="s">
-        <v>47</v>
-      </c>
-      <c r="I30" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J30" s="64"/>
-      <c r="K30" s="64"/>
-      <c r="L30" s="64"/>
-      <c r="M30" s="65"/>
+        <v>46</v>
+      </c>
+      <c r="I30" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J30" s="71"/>
+      <c r="K30" s="71"/>
+      <c r="L30" s="71"/>
+      <c r="M30" s="72"/>
       <c r="N30" s="35"/>
       <c r="O30" s="42"/>
     </row>
     <row r="31" spans="1:19" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="32"/>
       <c r="B31" s="33"/>
-      <c r="C31" s="57"/>
-      <c r="D31" s="58"/>
-      <c r="E31" s="58"/>
-      <c r="F31" s="59"/>
-      <c r="G31" s="60"/>
+      <c r="C31" s="47"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="48"/>
+      <c r="F31" s="49"/>
+      <c r="G31" s="50"/>
       <c r="H31" s="34"/>
-      <c r="I31" s="63"/>
-      <c r="J31" s="64"/>
-      <c r="K31" s="64"/>
-      <c r="L31" s="64"/>
-      <c r="M31" s="65"/>
+      <c r="I31" s="70"/>
+      <c r="J31" s="71"/>
+      <c r="K31" s="71"/>
+      <c r="L31" s="71"/>
+      <c r="M31" s="72"/>
       <c r="N31" s="35"/>
       <c r="O31" s="42"/>
     </row>
@@ -1861,250 +1861,250 @@
         <v>2</v>
       </c>
       <c r="B32" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="C32" s="51" t="s">
         <v>54</v>
       </c>
-      <c r="C32" s="67" t="s">
+      <c r="D32" s="52"/>
+      <c r="E32" s="52"/>
+      <c r="F32" s="53" t="s">
         <v>55</v>
       </c>
-      <c r="D32" s="55"/>
-      <c r="E32" s="55"/>
-      <c r="F32" s="72" t="s">
-        <v>56</v>
-      </c>
-      <c r="G32" s="73"/>
+      <c r="G32" s="54"/>
       <c r="H32" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="I32" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J32" s="64"/>
-      <c r="K32" s="64"/>
-      <c r="L32" s="64"/>
-      <c r="M32" s="65"/>
+        <v>38</v>
+      </c>
+      <c r="I32" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J32" s="71"/>
+      <c r="K32" s="71"/>
+      <c r="L32" s="71"/>
+      <c r="M32" s="72"/>
       <c r="N32" s="35" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="O32" s="42"/>
     </row>
     <row r="33" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="32"/>
       <c r="B33" s="33"/>
-      <c r="C33" s="57" t="s">
-        <v>26</v>
-      </c>
-      <c r="D33" s="58"/>
-      <c r="E33" s="58"/>
-      <c r="F33" s="70" t="s">
-        <v>56</v>
-      </c>
-      <c r="G33" s="71"/>
+      <c r="C33" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="D33" s="48"/>
+      <c r="E33" s="48"/>
+      <c r="F33" s="55" t="s">
+        <v>55</v>
+      </c>
+      <c r="G33" s="56"/>
       <c r="H33" s="34" t="s">
-        <v>40</v>
-      </c>
-      <c r="I33" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J33" s="64"/>
-      <c r="K33" s="64"/>
-      <c r="L33" s="64"/>
-      <c r="M33" s="65"/>
+        <v>39</v>
+      </c>
+      <c r="I33" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J33" s="71"/>
+      <c r="K33" s="71"/>
+      <c r="L33" s="71"/>
+      <c r="M33" s="72"/>
       <c r="N33" s="35" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="O33" s="42"/>
     </row>
     <row r="34" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="32"/>
       <c r="B34" s="33"/>
-      <c r="C34" s="61" t="s">
-        <v>29</v>
-      </c>
-      <c r="D34" s="62"/>
-      <c r="E34" s="62"/>
-      <c r="F34" s="68" t="s">
-        <v>56</v>
-      </c>
-      <c r="G34" s="69"/>
+      <c r="C34" s="57" t="s">
+        <v>28</v>
+      </c>
+      <c r="D34" s="58"/>
+      <c r="E34" s="58"/>
+      <c r="F34" s="59" t="s">
+        <v>55</v>
+      </c>
+      <c r="G34" s="60"/>
       <c r="H34" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="I34" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J34" s="64"/>
-      <c r="K34" s="64"/>
-      <c r="L34" s="64"/>
-      <c r="M34" s="65"/>
+        <v>40</v>
+      </c>
+      <c r="I34" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J34" s="71"/>
+      <c r="K34" s="71"/>
+      <c r="L34" s="71"/>
+      <c r="M34" s="72"/>
       <c r="N34" s="35" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="O34" s="42"/>
     </row>
     <row r="35" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="32"/>
       <c r="B35" s="33"/>
-      <c r="C35" s="57" t="s">
-        <v>28</v>
-      </c>
-      <c r="D35" s="58"/>
-      <c r="E35" s="58"/>
-      <c r="F35" s="59" t="s">
-        <v>56</v>
-      </c>
-      <c r="G35" s="60"/>
+      <c r="C35" s="47" t="s">
+        <v>27</v>
+      </c>
+      <c r="D35" s="48"/>
+      <c r="E35" s="48"/>
+      <c r="F35" s="49" t="s">
+        <v>55</v>
+      </c>
+      <c r="G35" s="50"/>
       <c r="H35" s="34" t="s">
-        <v>42</v>
-      </c>
-      <c r="I35" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J35" s="64"/>
-      <c r="K35" s="64"/>
-      <c r="L35" s="64"/>
-      <c r="M35" s="65"/>
+        <v>41</v>
+      </c>
+      <c r="I35" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J35" s="71"/>
+      <c r="K35" s="71"/>
+      <c r="L35" s="71"/>
+      <c r="M35" s="72"/>
       <c r="N35" s="35"/>
       <c r="O35" s="42"/>
     </row>
     <row r="36" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="32"/>
       <c r="B36" s="33"/>
-      <c r="C36" s="57"/>
-      <c r="D36" s="58"/>
-      <c r="E36" s="58"/>
-      <c r="F36" s="59"/>
-      <c r="G36" s="60"/>
+      <c r="C36" s="47"/>
+      <c r="D36" s="48"/>
+      <c r="E36" s="48"/>
+      <c r="F36" s="49"/>
+      <c r="G36" s="50"/>
       <c r="H36" s="34" t="s">
-        <v>43</v>
-      </c>
-      <c r="I36" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J36" s="64"/>
-      <c r="K36" s="64"/>
-      <c r="L36" s="64"/>
-      <c r="M36" s="65"/>
+        <v>42</v>
+      </c>
+      <c r="I36" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J36" s="71"/>
+      <c r="K36" s="71"/>
+      <c r="L36" s="71"/>
+      <c r="M36" s="72"/>
       <c r="N36" s="35"/>
       <c r="O36" s="42"/>
     </row>
     <row r="37" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="32"/>
       <c r="B37" s="33"/>
-      <c r="C37" s="57"/>
-      <c r="D37" s="58"/>
-      <c r="E37" s="58"/>
-      <c r="F37" s="59"/>
-      <c r="G37" s="60"/>
+      <c r="C37" s="47"/>
+      <c r="D37" s="48"/>
+      <c r="E37" s="48"/>
+      <c r="F37" s="49"/>
+      <c r="G37" s="50"/>
       <c r="H37" s="34" t="s">
-        <v>44</v>
-      </c>
-      <c r="I37" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J37" s="64"/>
-      <c r="K37" s="64"/>
-      <c r="L37" s="64"/>
-      <c r="M37" s="65"/>
+        <v>43</v>
+      </c>
+      <c r="I37" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J37" s="71"/>
+      <c r="K37" s="71"/>
+      <c r="L37" s="71"/>
+      <c r="M37" s="72"/>
       <c r="N37" s="35"/>
       <c r="O37" s="42"/>
     </row>
     <row r="38" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="32"/>
       <c r="B38" s="33"/>
-      <c r="C38" s="57"/>
-      <c r="D38" s="58"/>
-      <c r="E38" s="58"/>
-      <c r="F38" s="59"/>
-      <c r="G38" s="60"/>
+      <c r="C38" s="47"/>
+      <c r="D38" s="48"/>
+      <c r="E38" s="48"/>
+      <c r="F38" s="49"/>
+      <c r="G38" s="50"/>
       <c r="H38" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="I38" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J38" s="64"/>
-      <c r="K38" s="64"/>
-      <c r="L38" s="64"/>
-      <c r="M38" s="65"/>
+        <v>44</v>
+      </c>
+      <c r="I38" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J38" s="71"/>
+      <c r="K38" s="71"/>
+      <c r="L38" s="71"/>
+      <c r="M38" s="72"/>
       <c r="N38" s="35"/>
       <c r="O38" s="42"/>
     </row>
     <row r="39" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="32"/>
       <c r="B39" s="33"/>
-      <c r="C39" s="57"/>
-      <c r="D39" s="58"/>
-      <c r="E39" s="58"/>
-      <c r="F39" s="59"/>
-      <c r="G39" s="60"/>
+      <c r="C39" s="47"/>
+      <c r="D39" s="48"/>
+      <c r="E39" s="48"/>
+      <c r="F39" s="49"/>
+      <c r="G39" s="50"/>
       <c r="H39" s="34" t="s">
-        <v>46</v>
-      </c>
-      <c r="I39" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J39" s="64"/>
-      <c r="K39" s="64"/>
-      <c r="L39" s="64"/>
-      <c r="M39" s="65"/>
+        <v>45</v>
+      </c>
+      <c r="I39" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J39" s="71"/>
+      <c r="K39" s="71"/>
+      <c r="L39" s="71"/>
+      <c r="M39" s="72"/>
       <c r="N39" s="35"/>
       <c r="O39" s="42"/>
     </row>
     <row r="40" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="32"/>
       <c r="B40" s="33"/>
-      <c r="C40" s="57"/>
-      <c r="D40" s="58"/>
-      <c r="E40" s="58"/>
-      <c r="F40" s="59"/>
-      <c r="G40" s="60"/>
+      <c r="C40" s="47"/>
+      <c r="D40" s="48"/>
+      <c r="E40" s="48"/>
+      <c r="F40" s="49"/>
+      <c r="G40" s="50"/>
       <c r="H40" s="34" t="s">
-        <v>47</v>
-      </c>
-      <c r="I40" s="63" t="s">
-        <v>52</v>
-      </c>
-      <c r="J40" s="64"/>
-      <c r="K40" s="64"/>
-      <c r="L40" s="64"/>
-      <c r="M40" s="65"/>
+        <v>46</v>
+      </c>
+      <c r="I40" s="70" t="s">
+        <v>51</v>
+      </c>
+      <c r="J40" s="71"/>
+      <c r="K40" s="71"/>
+      <c r="L40" s="71"/>
+      <c r="M40" s="72"/>
       <c r="N40" s="35"/>
       <c r="O40" s="42"/>
     </row>
     <row r="41" spans="1:15" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="32"/>
       <c r="B41" s="33"/>
-      <c r="C41" s="57"/>
-      <c r="D41" s="58"/>
-      <c r="E41" s="58"/>
-      <c r="F41" s="59"/>
-      <c r="G41" s="60"/>
+      <c r="C41" s="47"/>
+      <c r="D41" s="48"/>
+      <c r="E41" s="48"/>
+      <c r="F41" s="49"/>
+      <c r="G41" s="50"/>
       <c r="H41" s="34"/>
-      <c r="I41" s="63"/>
-      <c r="J41" s="64"/>
-      <c r="K41" s="64"/>
-      <c r="L41" s="64"/>
-      <c r="M41" s="65"/>
+      <c r="I41" s="70"/>
+      <c r="J41" s="71"/>
+      <c r="K41" s="71"/>
+      <c r="L41" s="71"/>
+      <c r="M41" s="72"/>
       <c r="N41" s="35"/>
       <c r="O41" s="42"/>
     </row>
     <row r="42" spans="1:15" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B42" s="17"/>
-      <c r="C42" s="54"/>
-      <c r="D42" s="54"/>
-      <c r="E42" s="54"/>
-      <c r="F42" s="54"/>
-      <c r="G42" s="54"/>
-      <c r="H42" s="54"/>
-      <c r="I42" s="54"/>
-      <c r="J42" s="54"/>
-      <c r="K42" s="54"/>
-      <c r="L42" s="54"/>
-      <c r="M42" s="54"/>
-      <c r="N42" s="54"/>
+      <c r="C42" s="82"/>
+      <c r="D42" s="82"/>
+      <c r="E42" s="82"/>
+      <c r="F42" s="82"/>
+      <c r="G42" s="82"/>
+      <c r="H42" s="82"/>
+      <c r="I42" s="82"/>
+      <c r="J42" s="82"/>
+      <c r="K42" s="82"/>
+      <c r="L42" s="82"/>
+      <c r="M42" s="82"/>
+      <c r="N42" s="82"/>
       <c r="O42" s="12"/>
     </row>
     <row r="43" spans="1:15" ht="11.4" customHeight="1" x14ac:dyDescent="0.25">
@@ -2125,46 +2125,46 @@
       <c r="O43" s="17"/>
     </row>
     <row r="44" spans="1:15" ht="35.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="49" t="s">
-        <v>36</v>
-      </c>
-      <c r="B44" s="49"/>
-      <c r="C44" s="54">
+      <c r="A44" s="79" t="s">
+        <v>35</v>
+      </c>
+      <c r="B44" s="79"/>
+      <c r="C44" s="82">
         <f>+D13</f>
         <v>0</v>
       </c>
-      <c r="D44" s="54"/>
-      <c r="E44" s="54"/>
-      <c r="F44" s="54"/>
-      <c r="G44" s="54"/>
-      <c r="I44" s="75" t="s">
-        <v>37</v>
-      </c>
-      <c r="J44" s="75"/>
-      <c r="K44" s="76"/>
-      <c r="L44" s="76"/>
-      <c r="M44" s="76"/>
-      <c r="N44" s="76"/>
+      <c r="D44" s="82"/>
+      <c r="E44" s="82"/>
+      <c r="F44" s="82"/>
+      <c r="G44" s="82"/>
+      <c r="I44" s="73" t="s">
+        <v>36</v>
+      </c>
+      <c r="J44" s="73"/>
+      <c r="K44" s="74"/>
+      <c r="L44" s="74"/>
+      <c r="M44" s="74"/>
+      <c r="N44" s="74"/>
       <c r="O44" s="43"/>
     </row>
     <row r="45" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="1:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="47" t="s">
-        <v>57</v>
-      </c>
-      <c r="B46" s="47"/>
-      <c r="C46" s="47"/>
-      <c r="D46" s="47"/>
-      <c r="E46" s="47"/>
-      <c r="F46" s="47"/>
-      <c r="G46" s="47"/>
-      <c r="H46" s="47"/>
-      <c r="I46" s="47"/>
-      <c r="J46" s="47"/>
-      <c r="K46" s="47"/>
-      <c r="L46" s="47"/>
-      <c r="M46" s="47"/>
-      <c r="N46" s="47"/>
+      <c r="A46" s="77" t="s">
+        <v>56</v>
+      </c>
+      <c r="B46" s="77"/>
+      <c r="C46" s="77"/>
+      <c r="D46" s="77"/>
+      <c r="E46" s="77"/>
+      <c r="F46" s="77"/>
+      <c r="G46" s="77"/>
+      <c r="H46" s="77"/>
+      <c r="I46" s="77"/>
+      <c r="J46" s="77"/>
+      <c r="K46" s="77"/>
+      <c r="L46" s="77"/>
+      <c r="M46" s="77"/>
+      <c r="N46" s="77"/>
       <c r="O46" s="43"/>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
@@ -2178,79 +2178,6 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="89">
-    <mergeCell ref="C41:E41"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="C39:E39"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="I21:L21"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="E1:K4"/>
-    <mergeCell ref="K6:K7"/>
-    <mergeCell ref="D14:I14"/>
-    <mergeCell ref="K14:N14"/>
-    <mergeCell ref="D16:N16"/>
-    <mergeCell ref="D17:N17"/>
-    <mergeCell ref="D18:N18"/>
-    <mergeCell ref="D19:N19"/>
-    <mergeCell ref="I38:M38"/>
-    <mergeCell ref="I39:M39"/>
-    <mergeCell ref="I44:J44"/>
-    <mergeCell ref="K44:N44"/>
-    <mergeCell ref="I40:M40"/>
-    <mergeCell ref="I41:M41"/>
-    <mergeCell ref="I28:M28"/>
-    <mergeCell ref="I29:M29"/>
-    <mergeCell ref="I30:M30"/>
-    <mergeCell ref="I36:M36"/>
-    <mergeCell ref="I37:M37"/>
-    <mergeCell ref="I31:M31"/>
-    <mergeCell ref="I32:M32"/>
-    <mergeCell ref="I33:M33"/>
-    <mergeCell ref="I34:M34"/>
-    <mergeCell ref="I35:M35"/>
-    <mergeCell ref="I23:M23"/>
-    <mergeCell ref="I24:M24"/>
-    <mergeCell ref="I25:M25"/>
-    <mergeCell ref="I26:M26"/>
-    <mergeCell ref="I27:M27"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="A7:B7"/>
     <mergeCell ref="A46:N46"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A44:B44"/>
@@ -2267,6 +2194,79 @@
     <mergeCell ref="C24:E24"/>
     <mergeCell ref="C44:G44"/>
     <mergeCell ref="I22:M22"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="I23:M23"/>
+    <mergeCell ref="I24:M24"/>
+    <mergeCell ref="I25:M25"/>
+    <mergeCell ref="I26:M26"/>
+    <mergeCell ref="I27:M27"/>
+    <mergeCell ref="I28:M28"/>
+    <mergeCell ref="I29:M29"/>
+    <mergeCell ref="I30:M30"/>
+    <mergeCell ref="I36:M36"/>
+    <mergeCell ref="I37:M37"/>
+    <mergeCell ref="I31:M31"/>
+    <mergeCell ref="I32:M32"/>
+    <mergeCell ref="I33:M33"/>
+    <mergeCell ref="I34:M34"/>
+    <mergeCell ref="I35:M35"/>
+    <mergeCell ref="I38:M38"/>
+    <mergeCell ref="I39:M39"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="K44:N44"/>
+    <mergeCell ref="I40:M40"/>
+    <mergeCell ref="I41:M41"/>
+    <mergeCell ref="I21:L21"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="E1:K4"/>
+    <mergeCell ref="K6:K7"/>
+    <mergeCell ref="D14:I14"/>
+    <mergeCell ref="K14:N14"/>
+    <mergeCell ref="D16:N16"/>
+    <mergeCell ref="D17:N17"/>
+    <mergeCell ref="D18:N18"/>
+    <mergeCell ref="D19:N19"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="C41:E41"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="F39:G39"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>